<commit_message>
Kalkulačka: místo marginálního PNO „Na 100 Kč obratu navíc dáte“ v Kč
Srozumitelnější pro webinář: kolik Kč reklamy stojí 100 Kč obratu, které přinese navýšení.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plan-black-friday-kalkulacka.xlsx
+++ b/docs/plan-black-friday-kalkulacka.xlsx
@@ -18,7 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="d. m. yyyy"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -26,7 +26,8 @@
     <numFmt numFmtId="168" formatCode="0.00&quot;×&quot;"/>
     <numFmt numFmtId="169" formatCode="d. m."/>
     <numFmt numFmtId="170" formatCode="0.0%;-0.0%;&quot;-&quot;"/>
-    <numFmt numFmtId="171" formatCode="+0%;-0%;0%"/>
+    <numFmt numFmtId="171" formatCode="0.0&quot; Kč&quot;;-0.0&quot; Kč&quot;;&quot;-&quot;"/>
+    <numFmt numFmtId="172" formatCode="+0%;-0%;0%"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -154,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,19 +178,22 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1001,9 +1005,9 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
     <col width="52" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -1017,7 +1021,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ve žlutém sloupci „Úprava rozpočtu“ zkoušejte přidat nebo ubrat (např. 30 %). Hned uvidíte PNO týdne a jestli se navýšení vyplatí (marginální PNO proti marži).</t>
+          <t>Ve žlutém sloupci „Úprava rozpočtu“ zkoušejte přidat nebo ubrat (např. 30 %). Hned uvidíte PNO týdne a kolik vás stojí 100 Kč obratu, které přinese navýšení.</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1083,7 @@
       </c>
       <c r="L4" s="14" t="inlineStr">
         <is>
-          <t>Marginální PNO</t>
+          <t>Na 100 Kč obratu navíc dáte</t>
         </is>
       </c>
       <c r="M4" s="14" t="inlineStr">
@@ -1142,16 +1146,16 @@
         <f>IFERROR(I5/J5,"")</f>
         <v/>
       </c>
-      <c r="L5" s="19">
-        <f>IF(H5=0,"",IFERROR((I5-E5*Zadání!$B$21)/(J5-F5*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M5" s="21">
+      <c r="L5" s="21">
+        <f>IF(H5=0,"",IFERROR(100*(I5-E5*Zadání!$B$21)/(J5-F5*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M5" s="22">
         <f>IF(K5="","",IF(K5&gt;Zadání!$B$9,"prodělává",IF(K5&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N5" s="21">
-        <f>IF(H5&lt;=0,"",IF(L5="","",IF(L5&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
+      <c r="N5" s="22">
+        <f>IF(H5&lt;=0,"",IF(L5="","",IF(L5&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
         <v/>
       </c>
       <c r="O5" s="17" t="inlineStr">
@@ -1161,62 +1165,62 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="n">
+      <c r="A6" s="23" t="n">
         <v>46335</v>
       </c>
-      <c r="B6" s="23">
+      <c r="B6" s="24">
         <f>A6+6</f>
         <v/>
       </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C6" s="25" t="inlineStr">
         <is>
           <t>Rozjezd</t>
         </is>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="24">
         <f>A6-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E6" s="25">
+      <c r="E6" s="26">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D6)*(Data!$A$2:$A$3000&lt;=(D6+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F6" s="25">
+      <c r="F6" s="26">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D6)*(Data!$A$2:$A$3000&lt;=(D6+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
-      <c r="G6" s="26">
+      <c r="G6" s="27">
         <f>IFERROR(E6/F6,"")</f>
         <v/>
       </c>
       <c r="H6" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="25">
+      <c r="I6" s="26">
         <f>E6*Zadání!$B$21*(1+H6)</f>
         <v/>
       </c>
-      <c r="J6" s="25">
+      <c r="J6" s="26">
         <f>F6*Zadání!$B$22*(1+H6)^Zadání!$B$10</f>
         <v/>
       </c>
-      <c r="K6" s="26">
+      <c r="K6" s="27">
         <f>IFERROR(I6/J6,"")</f>
         <v/>
       </c>
-      <c r="L6" s="26">
-        <f>IF(H6=0,"",IFERROR((I6-E6*Zadání!$B$21)/(J6-F6*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M6" s="27">
+      <c r="L6" s="28">
+        <f>IF(H6=0,"",IFERROR(100*(I6-E6*Zadání!$B$21)/(J6-F6*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M6" s="29">
         <f>IF(K6="","",IF(K6&gt;Zadání!$B$9,"prodělává",IF(K6&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N6" s="27">
-        <f>IF(H6&lt;=0,"",IF(L6="","",IF(L6&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
-        <v/>
-      </c>
-      <c r="O6" s="24" t="inlineStr">
+      <c r="N6" s="29">
+        <f>IF(H6&lt;=0,"",IF(L6="","",IF(L6&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O6" s="25" t="inlineStr">
         <is>
           <t>Test 3 hooků na bannerech, plnit publika</t>
         </is>
@@ -1266,16 +1270,16 @@
         <f>IFERROR(I7/J7,"")</f>
         <v/>
       </c>
-      <c r="L7" s="19">
-        <f>IF(H7=0,"",IFERROR((I7-E7*Zadání!$B$21)/(J7-F7*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M7" s="21">
+      <c r="L7" s="21">
+        <f>IF(H7=0,"",IFERROR(100*(I7-E7*Zadání!$B$21)/(J7-F7*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M7" s="22">
         <f>IF(K7="","",IF(K7&gt;Zadání!$B$9,"prodělává",IF(K7&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N7" s="21">
-        <f>IF(H7&lt;=0,"",IF(L7="","",IF(L7&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
+      <c r="N7" s="22">
+        <f>IF(H7&lt;=0,"",IF(L7="","",IF(L7&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
         <v/>
       </c>
       <c r="O7" s="17" t="inlineStr">
@@ -1285,62 +1289,62 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="n">
+      <c r="A8" s="30" t="n">
         <v>46349</v>
       </c>
-      <c r="B8" s="29">
+      <c r="B8" s="31">
         <f>A8+6</f>
         <v/>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="C8" s="32" t="inlineStr">
         <is>
           <t>Black Week a Black Friday</t>
         </is>
       </c>
-      <c r="D8" s="29">
+      <c r="D8" s="31">
         <f>A8-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="33">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D8)*(Data!$A$2:$A$3000&lt;=(D8+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="33">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D8)*(Data!$A$2:$A$3000&lt;=(D8+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
-      <c r="G8" s="32">
+      <c r="G8" s="34">
         <f>IFERROR(E8/F8,"")</f>
         <v/>
       </c>
       <c r="H8" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="31">
+      <c r="I8" s="33">
         <f>E8*Zadání!$B$21*(1+H8)</f>
         <v/>
       </c>
-      <c r="J8" s="31">
+      <c r="J8" s="33">
         <f>F8*Zadání!$B$22*(1+H8)^Zadání!$B$10</f>
         <v/>
       </c>
-      <c r="K8" s="32">
+      <c r="K8" s="34">
         <f>IFERROR(I8/J8,"")</f>
         <v/>
       </c>
-      <c r="L8" s="32">
-        <f>IF(H8=0,"",IFERROR((I8-E8*Zadání!$B$21)/(J8-F8*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M8" s="33">
+      <c r="L8" s="35">
+        <f>IF(H8=0,"",IFERROR(100*(I8-E8*Zadání!$B$21)/(J8-F8*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M8" s="36">
         <f>IF(K8="","",IF(K8&gt;Zadání!$B$9,"prodělává",IF(K8&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N8" s="33">
-        <f>IF(H8&lt;=0,"",IF(L8="","",IF(L8&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
-        <v/>
-      </c>
-      <c r="O8" s="30" t="inlineStr">
+      <c r="N8" s="36">
+        <f>IF(H8&lt;=0,"",IF(L8="","",IF(L8&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O8" s="32" t="inlineStr">
         <is>
           <t>Rozpočty s rezervou, hlídat i večer a o víkendu</t>
         </is>
@@ -1390,16 +1394,16 @@
         <f>IFERROR(I9/J9,"")</f>
         <v/>
       </c>
-      <c r="L9" s="19">
-        <f>IF(H9=0,"",IFERROR((I9-E9*Zadání!$B$21)/(J9-F9*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M9" s="21">
+      <c r="L9" s="21">
+        <f>IF(H9=0,"",IFERROR(100*(I9-E9*Zadání!$B$21)/(J9-F9*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M9" s="22">
         <f>IF(K9="","",IF(K9&gt;Zadání!$B$9,"prodělává",IF(K9&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N9" s="21">
-        <f>IF(H9&lt;=0,"",IF(L9="","",IF(L9&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
+      <c r="N9" s="22">
+        <f>IF(H9&lt;=0,"",IF(L9="","",IF(L9&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
         <v/>
       </c>
       <c r="O9" s="17" t="inlineStr">
@@ -1409,62 +1413,62 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n">
+      <c r="A10" s="23" t="n">
         <v>46363</v>
       </c>
-      <c r="B10" s="23">
+      <c r="B10" s="24">
         <f>A10+6</f>
         <v/>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C10" s="25" t="inlineStr">
         <is>
           <t>Vánoční nákupy</t>
         </is>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="24">
         <f>A10-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E10" s="25">
+      <c r="E10" s="26">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D10)*(Data!$A$2:$A$3000&lt;=(D10+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F10" s="25">
+      <c r="F10" s="26">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D10)*(Data!$A$2:$A$3000&lt;=(D10+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
-      <c r="G10" s="26">
+      <c r="G10" s="27">
         <f>IFERROR(E10/F10,"")</f>
         <v/>
       </c>
       <c r="H10" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="25">
+      <c r="I10" s="26">
         <f>E10*Zadání!$B$21*(1+H10)</f>
         <v/>
       </c>
-      <c r="J10" s="25">
+      <c r="J10" s="26">
         <f>F10*Zadání!$B$22*(1+H10)^Zadání!$B$10</f>
         <v/>
       </c>
-      <c r="K10" s="26">
+      <c r="K10" s="27">
         <f>IFERROR(I10/J10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="26">
-        <f>IF(H10=0,"",IFERROR((I10-E10*Zadání!$B$21)/(J10-F10*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M10" s="27">
+      <c r="L10" s="28">
+        <f>IF(H10=0,"",IFERROR(100*(I10-E10*Zadání!$B$21)/(J10-F10*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M10" s="29">
         <f>IF(K10="","",IF(K10&gt;Zadání!$B$9,"prodělává",IF(K10&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N10" s="27">
-        <f>IF(H10&lt;=0,"",IF(L10="","",IF(L10&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
-        <v/>
-      </c>
-      <c r="O10" s="24" t="inlineStr">
+      <c r="N10" s="29">
+        <f>IF(H10&lt;=0,"",IF(L10="","",IF(L10&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O10" s="25" t="inlineStr">
         <is>
           <t>Dárkové kreativy, termín doručení</t>
         </is>
@@ -1514,16 +1518,16 @@
         <f>IFERROR(I11/J11,"")</f>
         <v/>
       </c>
-      <c r="L11" s="19">
-        <f>IF(H11=0,"",IFERROR((I11-E11*Zadání!$B$21)/(J11-F11*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M11" s="21">
+      <c r="L11" s="21">
+        <f>IF(H11=0,"",IFERROR(100*(I11-E11*Zadání!$B$21)/(J11-F11*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M11" s="22">
         <f>IF(K11="","",IF(K11&gt;Zadání!$B$9,"prodělává",IF(K11&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N11" s="21">
-        <f>IF(H11&lt;=0,"",IF(L11="","",IF(L11&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
+      <c r="N11" s="22">
+        <f>IF(H11&lt;=0,"",IF(L11="","",IF(L11&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
         <v/>
       </c>
       <c r="O11" s="17" t="inlineStr">
@@ -1533,62 +1537,62 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="n">
+      <c r="A12" s="23" t="n">
         <v>46377</v>
       </c>
-      <c r="B12" s="23">
+      <c r="B12" s="24">
         <f>A12+6</f>
         <v/>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="25" t="inlineStr">
         <is>
           <t>Po posledním doručení</t>
         </is>
       </c>
-      <c r="D12" s="23">
+      <c r="D12" s="24">
         <f>A12-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E12" s="25">
+      <c r="E12" s="26">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D12)*(Data!$A$2:$A$3000&lt;=(D12+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F12" s="25">
+      <c r="F12" s="26">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D12)*(Data!$A$2:$A$3000&lt;=(D12+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
-      <c r="G12" s="26">
+      <c r="G12" s="27">
         <f>IFERROR(E12/F12,"")</f>
         <v/>
       </c>
       <c r="H12" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="I12" s="25">
+      <c r="I12" s="26">
         <f>E12*Zadání!$B$21*(1+H12)</f>
         <v/>
       </c>
-      <c r="J12" s="25">
+      <c r="J12" s="26">
         <f>F12*Zadání!$B$22*(1+H12)^Zadání!$B$10</f>
         <v/>
       </c>
-      <c r="K12" s="26">
+      <c r="K12" s="27">
         <f>IFERROR(I12/J12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="26">
-        <f>IF(H12=0,"",IFERROR((I12-E12*Zadání!$B$21)/(J12-F12*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M12" s="27">
+      <c r="L12" s="28">
+        <f>IF(H12=0,"",IFERROR(100*(I12-E12*Zadání!$B$21)/(J12-F12*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M12" s="29">
         <f>IF(K12="","",IF(K12&gt;Zadání!$B$9,"prodělává",IF(K12&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N12" s="27">
-        <f>IF(H12&lt;=0,"",IF(L12="","",IF(L12&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
-        <v/>
-      </c>
-      <c r="O12" s="24" t="inlineStr">
+      <c r="N12" s="29">
+        <f>IF(H12&lt;=0,"",IF(L12="","",IF(L12&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O12" s="25" t="inlineStr">
         <is>
           <t>Ubrat, osobní odběr, dárkové poukazy</t>
         </is>
@@ -1638,16 +1642,16 @@
         <f>IFERROR(I13/J13,"")</f>
         <v/>
       </c>
-      <c r="L13" s="19">
-        <f>IF(H13=0,"",IFERROR((I13-E13*Zadání!$B$21)/(J13-F13*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M13" s="21">
+      <c r="L13" s="21">
+        <f>IF(H13=0,"",IFERROR(100*(I13-E13*Zadání!$B$21)/(J13-F13*Zadání!$B$22),""))</f>
+        <v/>
+      </c>
+      <c r="M13" s="22">
         <f>IF(K13="","",IF(K13&gt;Zadání!$B$9,"prodělává",IF(K13&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N13" s="21">
-        <f>IF(H13&lt;=0,"",IF(L13="","",IF(L13&gt;Zadání!$B$9,"přidaná koruna prodělává","vyplatí se")))</f>
+      <c r="N13" s="22">
+        <f>IF(H13&lt;=0,"",IF(L13="","",IF(L13&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
         <v/>
       </c>
       <c r="O13" s="17" t="inlineStr">
@@ -1657,53 +1661,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="34" t="inlineStr">
+      <c r="A14" s="37" t="inlineStr">
         <is>
           <t>Sezóna celkem</t>
         </is>
       </c>
-      <c r="B14" s="35" t="n"/>
-      <c r="C14" s="35" t="n"/>
-      <c r="D14" s="35" t="n"/>
-      <c r="E14" s="36">
+      <c r="B14" s="38" t="n"/>
+      <c r="C14" s="38" t="n"/>
+      <c r="D14" s="38" t="n"/>
+      <c r="E14" s="39">
         <f>SUM(E5:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="36">
+      <c r="F14" s="39">
         <f>SUM(F5:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="37">
+      <c r="G14" s="40">
         <f>IFERROR(E14/F14,"")</f>
         <v/>
       </c>
-      <c r="H14" s="35" t="n"/>
-      <c r="I14" s="36">
+      <c r="H14" s="38" t="n"/>
+      <c r="I14" s="39">
         <f>SUM(I5:I13)</f>
         <v/>
       </c>
-      <c r="J14" s="36">
+      <c r="J14" s="39">
         <f>SUM(J5:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="37">
+      <c r="K14" s="40">
         <f>IFERROR(I14/J14,"")</f>
         <v/>
       </c>
-      <c r="L14" s="35" t="n"/>
-      <c r="M14" s="35" t="n"/>
-      <c r="N14" s="35" t="n"/>
-      <c r="O14" s="35" t="n"/>
+      <c r="L14" s="38" t="n"/>
+      <c r="M14" s="38" t="n"/>
+      <c r="N14" s="38" t="n"/>
+      <c r="O14" s="38" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="38" t="inlineStr">
-        <is>
-          <t>Jak číst: Stav týdne = plánované PNO proti cíli a marži. Navýšení = marginální PNO, tedy kolik stojí koruna obratu navíc. Když přeleze marži, další peníze prodělávají, i když PNO týdne vypadá dobře.</t>
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>Jak číst: Stav týdne = plánované PNO proti cíli a marži. „Na 100 Kč obratu navíc dáte“ = kolik Kč reklamy stojí každých 100 Kč obratu, které přinese navýšení. Je to víc než marže? Navýšení prodělává, i když PNO týdne vypadá dobře.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="38" t="inlineStr">
+      <c r="A17" s="41" t="inlineStr">
         <is>
           <t>Je to odhad z historie, ne slib. Neví o slevách, skladu ani nových kampaních. Obrat = atribuce reklamních systémů, ne účetní tržba.</t>
         </is>
@@ -1738,71 +1742,71 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="39" t="inlineStr">
+      <c r="A1" s="42" t="inlineStr">
         <is>
           <t>Datum</t>
         </is>
       </c>
-      <c r="B1" s="39" t="inlineStr">
+      <c r="B1" s="42" t="inlineStr">
         <is>
           <t>Útrata (Kč, všechny systémy)</t>
         </is>
       </c>
-      <c r="C1" s="39" t="inlineStr">
+      <c r="C1" s="42" t="inlineStr">
         <is>
           <t>Obrat (Kč, všechny systémy)</t>
         </is>
       </c>
-      <c r="E1" s="40" t="inlineStr">
+      <c r="E1" s="43" t="inlineStr">
         <is>
           <t>Jak vyplnit</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="E2" s="41" t="inlineStr">
+      <c r="E2" s="44" t="inlineStr">
         <is>
           <t>Jeden řádek = jeden den, součet všech reklamních systémů (Google Ads + Sklik + Meta…).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="E3" s="41" t="inlineStr">
+      <c r="E3" s="44" t="inlineStr">
         <is>
           <t>Období: od 1. 9. loňského roku do včera. Datum jako datum (2025-09-01), čísla bez „Kč“.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E4" s="44" t="inlineStr">
         <is>
           <t>Příklad řádku: 1. 9. 2025 | 3 150 | 9 870</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="E5" s="41" t="inlineStr">
+      <c r="E5" s="44" t="inlineStr">
         <is>
           <t>Exporty po dnech: Google Ads (Den, Náklady, Hodnota konv.), Meta (Den, Utracená částka,</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="E6" s="41" t="inlineStr">
+      <c r="E6" s="44" t="inlineStr">
         <is>
           <t>Hodnota konverze nákupů), Sklik (Den, Cena, Hodnota konverzí). Dny ze systémů sečtěte.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="E7" s="41" t="inlineStr">
+      <c r="E7" s="44" t="inlineStr">
         <is>
           <t>Bez dat z reklam? Vložte do sloupce C tržby z GA4 a útratu nechte prázdnou: plán ukáže tvar sezóny.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="E8" s="41" t="inlineStr"/>
+      <c r="E8" s="44" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Kalkulačka: sloupec „Chci utratit“ místo procentní úpravy, tempo v % loňska
Letošní tempo je výchozí bod, ne strop. Uživatel napíše částku, kterou chce utratit,
a vidí odhad obratu, PNO a kolik stojí 100 Kč obratu navíc proti marži.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plan-black-friday-kalkulacka.xlsx
+++ b/docs/plan-black-friday-kalkulacka.xlsx
@@ -18,16 +18,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="d. m. yyyy"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; Kč&quot;;-#,##0&quot; Kč&quot;;&quot;-&quot;"/>
-    <numFmt numFmtId="168" formatCode="0.00&quot;×&quot;"/>
+    <numFmt numFmtId="168" formatCode="0%&quot; loňska&quot;"/>
     <numFmt numFmtId="169" formatCode="d. m."/>
     <numFmt numFmtId="170" formatCode="0.0%;-0.0%;&quot;-&quot;"/>
     <numFmt numFmtId="171" formatCode="0.0&quot; Kč&quot;;-0.0&quot; Kč&quot;;&quot;-&quot;"/>
-    <numFmt numFmtId="172" formatCode="+0%;-0%;0%"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -110,7 +109,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -125,6 +124,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="005924C6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C2187F"/>
       </patternFill>
     </fill>
     <fill>
@@ -155,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,28 +177,32 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="170" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="172" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="171" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="11" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -291,7 +299,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Plán útraty a obratu po týdnech</a:t>
+              <a:t>Chci utratit a odhad obratu po týdnech</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -412,9 +420,9 @@
     <author>PLACEMENT</author>
   </authors>
   <commentList>
-    <comment ref="H4" authorId="0" shapeId="0">
+    <comment ref="I4" authorId="0" shapeId="0">
       <text>
-        <t>Vyplňte: o kolik % chcete v týdnu rozpočet změnit proti loňsku × trend. Např. 30 % na Black Week.</t>
+        <t>Vyplňte: kolik Kč chcete v týdnu dát do reklamy. Předvyplněné je „jako teď“.</t>
       </text>
     </comment>
   </commentList>
@@ -427,7 +435,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>18</row>
+      <row>20</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -869,7 +877,7 @@
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
         <is>
-          <t>Trend: posledních 8 týdnů letos proti stejným 8 týdnům loni</t>
+          <t>Letošní tempo: posledních 8 týdnů letos proti stejným 8 týdnům loni</t>
         </is>
       </c>
     </row>
@@ -898,7 +906,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Trend útraty (letos / loni)</t>
+          <t>Útrata letos v % loňské</t>
         </is>
       </c>
       <c r="B15" s="12">
@@ -907,7 +915,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Pod 0,6× nebo nad 1,8× se účet nejspíš zásadně změnil. Zvažte vlastní trend níž.</t>
+          <t>Výchozí bod, ne strop: kolik vyjde, když pojedete jako teď. Z toho se bere, kolik obratu přináší koruna. Kolik chcete utratit, napíšete na listu Plán.</t>
         </is>
       </c>
     </row>
@@ -936,7 +944,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Trend obratu (letos / loni)</t>
+          <t>Obrat letos v % loňského</t>
         </is>
       </c>
       <c r="B18" s="12">
@@ -947,19 +955,19 @@
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
         <is>
-          <t>Vlastní trend (nechte prázdné = použije se spočítaný)</t>
+          <t>Vlastní tempo (nechte prázdné = použije se spočítané)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>← sem vlastní trend, např. 1,10 (kvůli novému systému nebo změně účtu)</t>
+          <t>← jen když se účet zásadně změnil (nový systém, jiné měření). Jinak nechte prázdné.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Trend útraty, který použijeme</t>
+          <t>Útrata v % loňské, se kterou počítáme</t>
         </is>
       </c>
       <c r="B21" s="12">
@@ -971,7 +979,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Trend obratu, který použijeme</t>
+          <t>Obrat v % loňského, se kterým počítáme</t>
         </is>
       </c>
       <c r="B22" s="12">
@@ -991,24 +999,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="52" customWidth="1" min="15" max="15"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1021,11 +1029,11 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ve žlutém sloupci „Úprava rozpočtu“ zkoušejte přidat nebo ubrat (např. 30 %). Hned uvidíte PNO týdne a kolik vás stojí 100 Kč obratu, které přinese navýšení.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
+          <t>Do žlutého sloupce „Chci utratit“ napište, kolik chcete v týdnu dát do reklamy (třeba 40 000). Hned uvidíte odhad obratu, PNO a jestli se peníze navíc vyplatí proti marži.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Týden od</t>
@@ -1058,27 +1066,27 @@
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>Loni PNO</t>
+          <t>Jako teď: útrata</t>
         </is>
       </c>
       <c r="H4" s="14" t="inlineStr">
         <is>
-          <t>Úprava rozpočtu</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>Plán útrata</t>
+          <t>Jako teď: obrat</t>
+        </is>
+      </c>
+      <c r="I4" s="15" t="inlineStr">
+        <is>
+          <t>Chci utratit</t>
         </is>
       </c>
       <c r="J4" s="14" t="inlineStr">
         <is>
-          <t>Plán obrat</t>
+          <t>Odhad obratu</t>
         </is>
       </c>
       <c r="K4" s="14" t="inlineStr">
         <is>
-          <t>Plán PNO</t>
+          <t>PNO</t>
         </is>
       </c>
       <c r="L4" s="14" t="inlineStr">
@@ -1103,611 +1111,637 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="n">
+      <c r="A5" s="16" t="n">
         <v>46328</v>
       </c>
-      <c r="B5" s="16">
+      <c r="B5" s="17">
         <f>A5+6</f>
         <v/>
       </c>
-      <c r="C5" s="17" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Rozjezd</t>
         </is>
       </c>
-      <c r="D5" s="16">
+      <c r="D5" s="17">
         <f>A5-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D5)*(Data!$A$2:$A$3000&lt;=(D5+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D5)*(Data!$A$2:$A$3000&lt;=(D5+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G5" s="19">
-        <f>IFERROR(E5/F5,"")</f>
-        <v/>
-      </c>
-      <c r="H5" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="18">
-        <f>E5*Zadání!$B$21*(1+H5)</f>
-        <v/>
-      </c>
-      <c r="J5" s="18">
-        <f>F5*Zadání!$B$22*(1+H5)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K5" s="19">
+        <f>E5*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H5" s="19">
+        <f>F5*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I5" s="20">
+        <f>ROUND(G5,-2)</f>
+        <v/>
+      </c>
+      <c r="J5" s="19">
+        <f>IF(G5&lt;=0,0,H5*(I5/G5)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K5" s="21">
         <f>IFERROR(I5/J5,"")</f>
         <v/>
       </c>
-      <c r="L5" s="21">
-        <f>IF(H5=0,"",IFERROR(100*(I5-E5*Zadání!$B$21)/(J5-F5*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M5" s="22">
+      <c r="L5" s="22">
+        <f>IF(ABS(I5-G5)&lt;100,"",IFERROR(100*(I5-G5)/(J5-H5),""))</f>
+        <v/>
+      </c>
+      <c r="M5" s="23">
         <f>IF(K5="","",IF(K5&gt;Zadání!$B$9,"prodělává",IF(K5&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N5" s="22">
-        <f>IF(H5&lt;=0,"",IF(L5="","",IF(L5&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O5" s="17" t="inlineStr">
+      <c r="N5" s="23">
+        <f>IF(L5="","",IF(I5&lt;G5,"ubráno",IF(L5&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O5" s="18" t="inlineStr">
         <is>
           <t>Teasery, early access, schválit BF kreativy</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
+      <c r="A6" s="24" t="n">
         <v>46335</v>
       </c>
-      <c r="B6" s="24">
+      <c r="B6" s="25">
         <f>A6+6</f>
         <v/>
       </c>
-      <c r="C6" s="25" t="inlineStr">
+      <c r="C6" s="26" t="inlineStr">
         <is>
           <t>Rozjezd</t>
         </is>
       </c>
-      <c r="D6" s="24">
+      <c r="D6" s="25">
         <f>A6-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="27">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D6)*(Data!$A$2:$A$3000&lt;=(D6+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="27">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D6)*(Data!$A$2:$A$3000&lt;=(D6+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G6" s="27">
-        <f>IFERROR(E6/F6,"")</f>
-        <v/>
-      </c>
-      <c r="H6" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="26">
-        <f>E6*Zadání!$B$21*(1+H6)</f>
-        <v/>
-      </c>
-      <c r="J6" s="26">
-        <f>F6*Zadání!$B$22*(1+H6)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K6" s="27">
+        <f>E6*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H6" s="27">
+        <f>F6*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I6" s="20">
+        <f>ROUND(G6,-2)</f>
+        <v/>
+      </c>
+      <c r="J6" s="27">
+        <f>IF(G6&lt;=0,0,H6*(I6/G6)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K6" s="28">
         <f>IFERROR(I6/J6,"")</f>
         <v/>
       </c>
-      <c r="L6" s="28">
-        <f>IF(H6=0,"",IFERROR(100*(I6-E6*Zadání!$B$21)/(J6-F6*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M6" s="29">
+      <c r="L6" s="29">
+        <f>IF(ABS(I6-G6)&lt;100,"",IFERROR(100*(I6-G6)/(J6-H6),""))</f>
+        <v/>
+      </c>
+      <c r="M6" s="30">
         <f>IF(K6="","",IF(K6&gt;Zadání!$B$9,"prodělává",IF(K6&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N6" s="29">
-        <f>IF(H6&lt;=0,"",IF(L6="","",IF(L6&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O6" s="25" t="inlineStr">
+      <c r="N6" s="30">
+        <f>IF(L6="","",IF(I6&lt;G6,"ubráno",IF(L6&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O6" s="26" t="inlineStr">
         <is>
           <t>Test 3 hooků na bannerech, plnit publika</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="n">
+      <c r="A7" s="16" t="n">
         <v>46342</v>
       </c>
-      <c r="B7" s="16">
+      <c r="B7" s="17">
         <f>A7+6</f>
         <v/>
       </c>
-      <c r="C7" s="17" t="inlineStr">
+      <c r="C7" s="18" t="inlineStr">
         <is>
           <t>Rozjezd → Black Week od 20. 11.</t>
         </is>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="17">
         <f>A7-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D7)*(Data!$A$2:$A$3000&lt;=(D7+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D7)*(Data!$A$2:$A$3000&lt;=(D7+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G7" s="19">
-        <f>IFERROR(E7/F7,"")</f>
-        <v/>
-      </c>
-      <c r="H7" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="18">
-        <f>E7*Zadání!$B$21*(1+H7)</f>
-        <v/>
-      </c>
-      <c r="J7" s="18">
-        <f>F7*Zadání!$B$22*(1+H7)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K7" s="19">
+        <f>E7*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H7" s="19">
+        <f>F7*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I7" s="20">
+        <f>ROUND(G7,-2)</f>
+        <v/>
+      </c>
+      <c r="J7" s="19">
+        <f>IF(G7&lt;=0,0,H7*(I7/G7)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K7" s="21">
         <f>IFERROR(I7/J7,"")</f>
         <v/>
       </c>
-      <c r="L7" s="21">
-        <f>IF(H7=0,"",IFERROR(100*(I7-E7*Zadání!$B$21)/(J7-F7*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M7" s="22">
+      <c r="L7" s="22">
+        <f>IF(ABS(I7-G7)&lt;100,"",IFERROR(100*(I7-G7)/(J7-H7),""))</f>
+        <v/>
+      </c>
+      <c r="M7" s="23">
         <f>IF(K7="","",IF(K7&gt;Zadání!$B$9,"prodělává",IF(K7&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N7" s="22">
-        <f>IF(H7&lt;=0,"",IF(L7="","",IF(L7&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O7" s="17" t="inlineStr">
+      <c r="N7" s="23">
+        <f>IF(L7="","",IF(I7&lt;G7,"ubráno",IF(L7&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O7" s="18" t="inlineStr">
         <is>
           <t>Spustit nabídku, zpřísnit hlídač</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="n">
+      <c r="A8" s="31" t="n">
         <v>46349</v>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="32">
         <f>A8+6</f>
         <v/>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>Black Week a Black Friday</t>
         </is>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="32">
         <f>A8-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E8" s="33">
+      <c r="E8" s="34">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D8)*(Data!$A$2:$A$3000&lt;=(D8+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="34">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D8)*(Data!$A$2:$A$3000&lt;=(D8+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G8" s="34">
-        <f>IFERROR(E8/F8,"")</f>
-        <v/>
-      </c>
-      <c r="H8" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" s="33">
-        <f>E8*Zadání!$B$21*(1+H8)</f>
-        <v/>
-      </c>
-      <c r="J8" s="33">
-        <f>F8*Zadání!$B$22*(1+H8)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K8" s="34">
+        <f>E8*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H8" s="34">
+        <f>F8*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I8" s="35">
+        <f>ROUND(G8,-2)</f>
+        <v/>
+      </c>
+      <c r="J8" s="34">
+        <f>IF(G8&lt;=0,0,H8*(I8/G8)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K8" s="36">
         <f>IFERROR(I8/J8,"")</f>
         <v/>
       </c>
-      <c r="L8" s="35">
-        <f>IF(H8=0,"",IFERROR(100*(I8-E8*Zadání!$B$21)/(J8-F8*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M8" s="36">
+      <c r="L8" s="37">
+        <f>IF(ABS(I8-G8)&lt;100,"",IFERROR(100*(I8-G8)/(J8-H8),""))</f>
+        <v/>
+      </c>
+      <c r="M8" s="38">
         <f>IF(K8="","",IF(K8&gt;Zadání!$B$9,"prodělává",IF(K8&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N8" s="36">
-        <f>IF(H8&lt;=0,"",IF(L8="","",IF(L8&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O8" s="32" t="inlineStr">
+      <c r="N8" s="38">
+        <f>IF(L8="","",IF(I8&lt;G8,"ubráno",IF(L8&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O8" s="33" t="inlineStr">
         <is>
           <t>Rozpočty s rezervou, hlídat i večer a o víkendu</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="n">
+      <c r="A9" s="16" t="n">
         <v>46356</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="17">
         <f>A9+6</f>
         <v/>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Cyber Monday, pak Vánoce</t>
         </is>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="17">
         <f>A9-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D9)*(Data!$A$2:$A$3000&lt;=(D9+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D9)*(Data!$A$2:$A$3000&lt;=(D9+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G9" s="19">
-        <f>IFERROR(E9/F9,"")</f>
-        <v/>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="18">
-        <f>E9*Zadání!$B$21*(1+H9)</f>
-        <v/>
-      </c>
-      <c r="J9" s="18">
-        <f>F9*Zadání!$B$22*(1+H9)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K9" s="19">
+        <f>E9*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H9" s="19">
+        <f>F9*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I9" s="20">
+        <f>ROUND(G9,-2)</f>
+        <v/>
+      </c>
+      <c r="J9" s="19">
+        <f>IF(G9&lt;=0,0,H9*(I9/G9)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K9" s="21">
         <f>IFERROR(I9/J9,"")</f>
         <v/>
       </c>
-      <c r="L9" s="21">
-        <f>IF(H9=0,"",IFERROR(100*(I9-E9*Zadání!$B$21)/(J9-F9*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M9" s="22">
+      <c r="L9" s="22">
+        <f>IF(ABS(I9-G9)&lt;100,"",IFERROR(100*(I9-G9)/(J9-H9),""))</f>
+        <v/>
+      </c>
+      <c r="M9" s="23">
         <f>IF(K9="","",IF(K9&gt;Zadání!$B$9,"prodělává",IF(K9&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N9" s="22">
-        <f>IF(H9&lt;=0,"",IF(L9="","",IF(L9&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O9" s="17" t="inlineStr">
+      <c r="N9" s="23">
+        <f>IF(L9="","",IF(I9&lt;G9,"ubráno",IF(L9&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O9" s="18" t="inlineStr">
         <is>
           <t>Poslední den akce, přepnout na dárky</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
+      <c r="A10" s="24" t="n">
         <v>46363</v>
       </c>
-      <c r="B10" s="24">
+      <c r="B10" s="25">
         <f>A10+6</f>
         <v/>
       </c>
-      <c r="C10" s="25" t="inlineStr">
+      <c r="C10" s="26" t="inlineStr">
         <is>
           <t>Vánoční nákupy</t>
         </is>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="25">
         <f>A10-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="27">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D10)*(Data!$A$2:$A$3000&lt;=(D10+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="27">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D10)*(Data!$A$2:$A$3000&lt;=(D10+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G10" s="27">
-        <f>IFERROR(E10/F10,"")</f>
-        <v/>
-      </c>
-      <c r="H10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="26">
-        <f>E10*Zadání!$B$21*(1+H10)</f>
-        <v/>
-      </c>
-      <c r="J10" s="26">
-        <f>F10*Zadání!$B$22*(1+H10)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K10" s="27">
+        <f>E10*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H10" s="27">
+        <f>F10*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I10" s="20">
+        <f>ROUND(G10,-2)</f>
+        <v/>
+      </c>
+      <c r="J10" s="27">
+        <f>IF(G10&lt;=0,0,H10*(I10/G10)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="28">
         <f>IFERROR(I10/J10,"")</f>
         <v/>
       </c>
-      <c r="L10" s="28">
-        <f>IF(H10=0,"",IFERROR(100*(I10-E10*Zadání!$B$21)/(J10-F10*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M10" s="29">
+      <c r="L10" s="29">
+        <f>IF(ABS(I10-G10)&lt;100,"",IFERROR(100*(I10-G10)/(J10-H10),""))</f>
+        <v/>
+      </c>
+      <c r="M10" s="30">
         <f>IF(K10="","",IF(K10&gt;Zadání!$B$9,"prodělává",IF(K10&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N10" s="29">
-        <f>IF(H10&lt;=0,"",IF(L10="","",IF(L10&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O10" s="25" t="inlineStr">
+      <c r="N10" s="30">
+        <f>IF(L10="","",IF(I10&lt;G10,"ubráno",IF(L10&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O10" s="26" t="inlineStr">
         <is>
           <t>Dárkové kreativy, termín doručení</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="n">
+      <c r="A11" s="16" t="n">
         <v>46370</v>
       </c>
-      <c r="B11" s="16">
+      <c r="B11" s="17">
         <f>A11+6</f>
         <v/>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>Vánoční nákupy, doručení do 18. 12.</t>
         </is>
       </c>
-      <c r="D11" s="16">
+      <c r="D11" s="17">
         <f>A11-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D11)*(Data!$A$2:$A$3000&lt;=(D11+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D11)*(Data!$A$2:$A$3000&lt;=(D11+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G11" s="19">
-        <f>IFERROR(E11/F11,"")</f>
-        <v/>
-      </c>
-      <c r="H11" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="18">
-        <f>E11*Zadání!$B$21*(1+H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="18">
-        <f>F11*Zadání!$B$22*(1+H11)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K11" s="19">
+        <f>E11*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H11" s="19">
+        <f>F11*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I11" s="20">
+        <f>ROUND(G11,-2)</f>
+        <v/>
+      </c>
+      <c r="J11" s="19">
+        <f>IF(G11&lt;=0,0,H11*(I11/G11)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K11" s="21">
         <f>IFERROR(I11/J11,"")</f>
         <v/>
       </c>
-      <c r="L11" s="21">
-        <f>IF(H11=0,"",IFERROR(100*(I11-E11*Zadání!$B$21)/(J11-F11*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M11" s="22">
+      <c r="L11" s="22">
+        <f>IF(ABS(I11-G11)&lt;100,"",IFERROR(100*(I11-G11)/(J11-H11),""))</f>
+        <v/>
+      </c>
+      <c r="M11" s="23">
         <f>IF(K11="","",IF(K11&gt;Zadání!$B$9,"prodělává",IF(K11&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N11" s="22">
-        <f>IF(H11&lt;=0,"",IF(L11="","",IF(L11&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O11" s="17" t="inlineStr">
+      <c r="N11" s="23">
+        <f>IF(L11="","",IF(I11&lt;G11,"ubráno",IF(L11&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O11" s="18" t="inlineStr">
         <is>
           <t>Hlídat sklad top produktů</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="24" t="n">
         <v>46377</v>
       </c>
-      <c r="B12" s="24">
+      <c r="B12" s="25">
         <f>A12+6</f>
         <v/>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>Po posledním doručení</t>
         </is>
       </c>
-      <c r="D12" s="24">
+      <c r="D12" s="25">
         <f>A12-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="27">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D12)*(Data!$A$2:$A$3000&lt;=(D12+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="27">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D12)*(Data!$A$2:$A$3000&lt;=(D12+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G12" s="27">
-        <f>IFERROR(E12/F12,"")</f>
-        <v/>
-      </c>
-      <c r="H12" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="26">
-        <f>E12*Zadání!$B$21*(1+H12)</f>
-        <v/>
-      </c>
-      <c r="J12" s="26">
-        <f>F12*Zadání!$B$22*(1+H12)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K12" s="27">
+        <f>E12*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H12" s="27">
+        <f>F12*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I12" s="20">
+        <f>ROUND(G12,-2)</f>
+        <v/>
+      </c>
+      <c r="J12" s="27">
+        <f>IF(G12&lt;=0,0,H12*(I12/G12)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K12" s="28">
         <f>IFERROR(I12/J12,"")</f>
         <v/>
       </c>
-      <c r="L12" s="28">
-        <f>IF(H12=0,"",IFERROR(100*(I12-E12*Zadání!$B$21)/(J12-F12*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M12" s="29">
+      <c r="L12" s="29">
+        <f>IF(ABS(I12-G12)&lt;100,"",IFERROR(100*(I12-G12)/(J12-H12),""))</f>
+        <v/>
+      </c>
+      <c r="M12" s="30">
         <f>IF(K12="","",IF(K12&gt;Zadání!$B$9,"prodělává",IF(K12&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N12" s="29">
-        <f>IF(H12&lt;=0,"",IF(L12="","",IF(L12&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O12" s="25" t="inlineStr">
+      <c r="N12" s="30">
+        <f>IF(L12="","",IF(I12&lt;G12,"ubráno",IF(L12&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O12" s="26" t="inlineStr">
         <is>
           <t>Ubrat, osobní odběr, dárkové poukazy</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="n">
+      <c r="A13" s="16" t="n">
         <v>46384</v>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="17">
         <f>A13+6</f>
         <v/>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr">
         <is>
           <t>Po Vánocích</t>
         </is>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="17">
         <f>A13-Zadání!$B$6</f>
         <v/>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D13)*(Data!$A$2:$A$3000&lt;=(D13+6))*Data!$B$2:$B$3000)</f>
         <v/>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="19">
         <f>SUMPRODUCT((Data!$A$2:$A$3000&gt;=D13)*(Data!$A$2:$A$3000&lt;=(D13+6))*Data!$C$2:$C$3000)</f>
         <v/>
       </c>
       <c r="G13" s="19">
-        <f>IFERROR(E13/F13,"")</f>
-        <v/>
-      </c>
-      <c r="H13" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="18">
-        <f>E13*Zadání!$B$21*(1+H13)</f>
-        <v/>
-      </c>
-      <c r="J13" s="18">
-        <f>F13*Zadání!$B$22*(1+H13)^Zadání!$B$10</f>
-        <v/>
-      </c>
-      <c r="K13" s="19">
+        <f>E13*Zadání!$B$21</f>
+        <v/>
+      </c>
+      <c r="H13" s="19">
+        <f>F13*Zadání!$B$22</f>
+        <v/>
+      </c>
+      <c r="I13" s="20">
+        <f>ROUND(G13,-2)</f>
+        <v/>
+      </c>
+      <c r="J13" s="19">
+        <f>IF(G13&lt;=0,0,H13*(I13/G13)^Zadání!$B$10)</f>
+        <v/>
+      </c>
+      <c r="K13" s="21">
         <f>IFERROR(I13/J13,"")</f>
         <v/>
       </c>
-      <c r="L13" s="21">
-        <f>IF(H13=0,"",IFERROR(100*(I13-E13*Zadání!$B$21)/(J13-F13*Zadání!$B$22),""))</f>
-        <v/>
-      </c>
-      <c r="M13" s="22">
+      <c r="L13" s="22">
+        <f>IF(ABS(I13-G13)&lt;100,"",IFERROR(100*(I13-G13)/(J13-H13),""))</f>
+        <v/>
+      </c>
+      <c r="M13" s="23">
         <f>IF(K13="","",IF(K13&gt;Zadání!$B$9,"prodělává",IF(K13&gt;Zadání!$B$8,"nad cílem","v cíli")))</f>
         <v/>
       </c>
-      <c r="N13" s="22">
-        <f>IF(H13&lt;=0,"",IF(L13="","",IF(L13&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
-        <v/>
-      </c>
-      <c r="O13" s="17" t="inlineStr">
+      <c r="N13" s="23">
+        <f>IF(L13="","",IF(I13&lt;G13,"ubráno",IF(L13&gt;100*Zadání!$B$9,"navýšení prodělává","navýšení vydělá")))</f>
+        <v/>
+      </c>
+      <c r="O13" s="18" t="inlineStr">
         <is>
           <t>Výprodej, vyhodnotit sezónu</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="37" t="inlineStr">
+      <c r="A14" s="39" t="inlineStr">
         <is>
           <t>Sezóna celkem</t>
         </is>
       </c>
-      <c r="B14" s="38" t="n"/>
-      <c r="C14" s="38" t="n"/>
-      <c r="D14" s="38" t="n"/>
-      <c r="E14" s="39">
+      <c r="B14" s="40" t="n"/>
+      <c r="C14" s="40" t="n"/>
+      <c r="D14" s="40" t="n"/>
+      <c r="E14" s="41">
         <f>SUM(E5:E13)</f>
         <v/>
       </c>
-      <c r="F14" s="39">
+      <c r="F14" s="41">
         <f>SUM(F5:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="40">
-        <f>IFERROR(E14/F14,"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="38" t="n"/>
-      <c r="I14" s="39">
+      <c r="G14" s="41">
+        <f>SUM(G5:G13)</f>
+        <v/>
+      </c>
+      <c r="H14" s="41">
+        <f>SUM(H5:H13)</f>
+        <v/>
+      </c>
+      <c r="I14" s="41">
         <f>SUM(I5:I13)</f>
         <v/>
       </c>
-      <c r="J14" s="39">
+      <c r="J14" s="41">
         <f>SUM(J5:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="40">
+      <c r="K14" s="42">
         <f>IFERROR(I14/J14,"")</f>
         <v/>
       </c>
-      <c r="L14" s="38" t="n"/>
-      <c r="M14" s="38" t="n"/>
-      <c r="N14" s="38" t="n"/>
-      <c r="O14" s="38" t="n"/>
+      <c r="L14" s="40" t="n"/>
+      <c r="M14" s="40" t="n"/>
+      <c r="N14" s="40" t="n"/>
+      <c r="O14" s="40" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="41" t="inlineStr">
-        <is>
-          <t>Jak číst: Stav týdne = plánované PNO proti cíli a marži. „Na 100 Kč obratu navíc dáte“ = kolik Kč reklamy stojí každých 100 Kč obratu, které přinese navýšení. Je to víc než marže? Navýšení prodělává, i když PNO týdne vypadá dobře.</t>
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>„Jako teď“ = loňský týden přepočtený na letošní tempo (list Zadání). Výchozí bod, ne strop.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="41" t="inlineStr">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>„Chci utratit“ = vaše rozhodnutí. Obrat neroste stejně rychle jako útrata: +10 % útraty ≈ +6 % obratu (list Zadání, upravitelné).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>„Na 100 Kč obratu navíc dáte“ = kolik Kč reklamy stojí každých 100 Kč obratu, které přinesou peníze navíc. Víc než marže? Navýšení prodělává, i když PNO týdne vypadá dobře.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="43" t="inlineStr">
         <is>
           <t>Je to odhad z historie, ne slib. Neví o slevách, skladu ani nových kampaních. Obrat = atribuce reklamních systémů, ne účetní tržba.</t>
         </is>
@@ -1715,9 +1749,8 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="between">
-      <formula1>-1</formula1>
-      <formula2>3</formula2>
+    <dataValidation sqref="I5:I13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1742,71 +1775,71 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="42" t="inlineStr">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>Datum</t>
         </is>
       </c>
-      <c r="B1" s="42" t="inlineStr">
+      <c r="B1" s="44" t="inlineStr">
         <is>
           <t>Útrata (Kč, všechny systémy)</t>
         </is>
       </c>
-      <c r="C1" s="42" t="inlineStr">
+      <c r="C1" s="44" t="inlineStr">
         <is>
           <t>Obrat (Kč, všechny systémy)</t>
         </is>
       </c>
-      <c r="E1" s="43" t="inlineStr">
+      <c r="E1" s="45" t="inlineStr">
         <is>
           <t>Jak vyplnit</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="E2" s="44" t="inlineStr">
+      <c r="E2" s="46" t="inlineStr">
         <is>
           <t>Jeden řádek = jeden den, součet všech reklamních systémů (Google Ads + Sklik + Meta…).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="E3" s="44" t="inlineStr">
+      <c r="E3" s="46" t="inlineStr">
         <is>
           <t>Období: od 1. 9. loňského roku do včera. Datum jako datum (2025-09-01), čísla bez „Kč“.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="E4" s="44" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>Příklad řádku: 1. 9. 2025 | 3 150 | 9 870</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="E5" s="44" t="inlineStr">
+      <c r="E5" s="46" t="inlineStr">
         <is>
           <t>Exporty po dnech: Google Ads (Den, Náklady, Hodnota konv.), Meta (Den, Utracená částka,</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="E6" s="44" t="inlineStr">
+      <c r="E6" s="46" t="inlineStr">
         <is>
           <t>Hodnota konverze nákupů), Sklik (Den, Cena, Hodnota konverzí). Dny ze systémů sečtěte.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="E7" s="44" t="inlineStr">
+      <c r="E7" s="46" t="inlineStr">
         <is>
           <t>Bez dat z reklam? Vložte do sloupce C tržby z GA4 a útratu nechte prázdnou: plán ukáže tvar sezóny.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="E8" s="44" t="inlineStr"/>
+      <c r="E8" s="46" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Kalkulačka: neutrální výchozí cíl a marže (25 % / 40 %), prompt na rozhýbání bez závislosti na lokální složce
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/plan-black-friday-kalkulacka.xlsx
+++ b/docs/plan-black-friday-kalkulacka.xlsx
@@ -836,11 +836,11 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>0.52</v>
+        <v>0.25</v>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Náklady / obrat. Cíl ROAS 190 % = PNO 52,6 %.</t>
+          <t>Náklady / obrat. Doplňte svůj cíl (ROAS 400 % = PNO 25 %).</t>
         </is>
       </c>
     </row>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>0.495</v>
+        <v>0.4</v>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>

</xml_diff>